<commit_message>
v5.778 — template-retro.xlsx: aggiunte colonne "Errore di stampa" e "Tipo di errore di stampa" (chiude DA FARE #1); nota di processo consegna nel changelog
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YuXK6if3H6iVAZ3AUavow
</commit_message>
<xml_diff>
--- a/templates/template-retro.xlsx
+++ b/templates/template-retro.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -434,8 +434,10 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -461,15 +463,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Errore di stampa</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Tipo di change</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo di errore di stampa</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Retro - Categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Retro - Nome</t>
         </is>

</xml_diff>